<commit_message>
fixed graphs and UI improvement
</commit_message>
<xml_diff>
--- a/measurements/report.xlsx
+++ b/measurements/report.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kamil\Documents\TUKE\TUKE_skola\ING\1.rocnik\LS\PPS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kamil\Documents\TUKE\TUKE_skola\ING\1.rocnik\LS\PPS\Parallel-Computer-Systems---assignment\3-volitelna\measurements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36DB43DC-A973-48CC-AE35-DDE7AF2CFA84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A364557E-1341-43B6-8026-06F3318A58DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{7107CA0B-3E53-4ED7-B3BD-8029C5150CF5}"/>
+    <workbookView xWindow="1710" yWindow="-14490" windowWidth="21600" windowHeight="11175" xr2:uid="{7107CA0B-3E53-4ED7-B3BD-8029C5150CF5}"/>
   </bookViews>
   <sheets>
     <sheet name="3-volitelna" sheetId="1" r:id="rId1"/>
@@ -736,6 +736,99 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -771,99 +864,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5387,19 +5387,19 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.49066390041493774</c:v>
+                  <c:v>0.98132780082987547</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.41932624113475181</c:v>
+                  <c:v>0.83865248226950362</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.51864035087719296</c:v>
+                  <c:v>0.77796052631578949</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.48463114754098358</c:v>
+                  <c:v>0.64617486338797814</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.51864035087719296</c:v>
+                  <c:v>0.69152046783625731</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6585,16 +6585,16 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.49116347569955815</c:v>
+                  <c:v>0.9823269513991163</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.45128552097428959</c:v>
+                  <c:v>0.90257104194857918</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.5409570154095702</c:v>
+                  <c:v>0.81143552311435529</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.53964401294498388</c:v>
+                  <c:v>0.7195253505933118</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0.64382239382239381</c:v>
@@ -7776,16 +7776,16 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.51631557207765388</c:v>
+                  <c:v>1.0326311441553078</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.48262548262548266</c:v>
+                  <c:v>0.96525096525096532</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.5376344086021505</c:v>
+                  <c:v>0.80645161290322576</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.56205035971223016</c:v>
+                  <c:v>0.74940047961630685</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0.62877263581488929</c:v>
@@ -8974,16 +8974,16 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.48798743300683795</c:v>
+                  <c:v>0.97597486601367589</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.46259635599159071</c:v>
+                  <c:v>0.92519271198318143</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.53898754847928143</c:v>
+                  <c:v>0.80848132271892215</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.56085386576040774</c:v>
+                  <c:v>0.74780515434721029</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0.66814271255060731</c:v>
@@ -14620,66 +14620,66 @@
   <sheetData>
     <row r="2" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="84" t="s">
+      <c r="B3" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="85"/>
-      <c r="D3" s="85"/>
-      <c r="E3" s="85"/>
-      <c r="F3" s="85"/>
-      <c r="G3" s="85"/>
-      <c r="H3" s="85"/>
-      <c r="I3" s="85"/>
-      <c r="J3" s="85"/>
-      <c r="K3" s="85"/>
-      <c r="L3" s="85"/>
-      <c r="M3" s="85"/>
-      <c r="N3" s="86"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="45"/>
+      <c r="I3" s="45"/>
+      <c r="J3" s="45"/>
+      <c r="K3" s="45"/>
+      <c r="L3" s="45"/>
+      <c r="M3" s="45"/>
+      <c r="N3" s="46"/>
     </row>
     <row r="4" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="59" t="s">
+      <c r="B4" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="62" t="s">
+      <c r="C4" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="63"/>
-      <c r="L4" s="63"/>
-      <c r="M4" s="63"/>
-      <c r="N4" s="64"/>
+      <c r="D4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="51"/>
+      <c r="G4" s="51"/>
+      <c r="H4" s="51"/>
+      <c r="I4" s="51"/>
+      <c r="J4" s="51"/>
+      <c r="K4" s="51"/>
+      <c r="L4" s="51"/>
+      <c r="M4" s="51"/>
+      <c r="N4" s="52"/>
     </row>
     <row r="5" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="81"/>
-      <c r="C5" s="65">
+      <c r="B5" s="48"/>
+      <c r="C5" s="53">
         <v>500</v>
       </c>
-      <c r="D5" s="66"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="68">
+      <c r="D5" s="54"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="56">
         <v>1000</v>
       </c>
-      <c r="G5" s="69"/>
-      <c r="H5" s="70"/>
-      <c r="I5" s="65">
+      <c r="G5" s="57"/>
+      <c r="H5" s="58"/>
+      <c r="I5" s="53">
         <v>2000</v>
       </c>
-      <c r="J5" s="66"/>
-      <c r="K5" s="67"/>
-      <c r="L5" s="68">
+      <c r="J5" s="54"/>
+      <c r="K5" s="55"/>
+      <c r="L5" s="56">
         <v>5000</v>
       </c>
-      <c r="M5" s="69"/>
-      <c r="N5" s="70"/>
+      <c r="M5" s="57"/>
+      <c r="N5" s="58"/>
     </row>
     <row r="6" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="82"/>
+      <c r="B6" s="49"/>
       <c r="C6" s="2" t="s">
         <v>3</v>
       </c>
@@ -14797,8 +14797,8 @@
         <v>1.9626556016597509</v>
       </c>
       <c r="K8" s="12">
-        <f xml:space="preserve"> J8 / 4</f>
-        <v>0.49066390041493774</v>
+        <f xml:space="preserve"> J8 / 2</f>
+        <v>0.98132780082987547</v>
       </c>
       <c r="L8" s="10">
         <v>0.59599999999999997</v>
@@ -14846,8 +14846,8 @@
         <v>3.3546099290780145</v>
       </c>
       <c r="K9" s="16">
-        <f xml:space="preserve"> J9 / 8</f>
-        <v>0.41932624113475181</v>
+        <f xml:space="preserve"> J9 / 4</f>
+        <v>0.83865248226950362</v>
       </c>
       <c r="L9" s="14">
         <v>0.32200000000000001</v>
@@ -14895,8 +14895,8 @@
         <v>6.2236842105263159</v>
       </c>
       <c r="K10" s="12">
-        <f xml:space="preserve"> J10 / 12</f>
-        <v>0.51864035087719296</v>
+        <f xml:space="preserve"> J10 / 8</f>
+        <v>0.77796052631578949</v>
       </c>
       <c r="L10" s="10">
         <v>0.19600000000000001</v>
@@ -14944,8 +14944,8 @@
         <v>7.7540983606557372</v>
       </c>
       <c r="K11" s="16">
-        <f xml:space="preserve"> J11 / 16</f>
-        <v>0.48463114754098358</v>
+        <f xml:space="preserve"> J11 / 12</f>
+        <v>0.64617486338797814</v>
       </c>
       <c r="L11" s="14">
         <v>0.151</v>
@@ -14993,8 +14993,8 @@
         <v>8.2982456140350873</v>
       </c>
       <c r="K12" s="20">
-        <f xml:space="preserve"> J12 / 16</f>
-        <v>0.51864035087719296</v>
+        <f xml:space="preserve"> J12 / 12</f>
+        <v>0.69152046783625731</v>
       </c>
       <c r="L12" s="18">
         <v>0.14000000000000001</v>
@@ -15010,66 +15010,66 @@
     </row>
     <row r="13" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="14" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="78" t="s">
+      <c r="B14" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="79"/>
-      <c r="D14" s="79"/>
-      <c r="E14" s="79"/>
-      <c r="F14" s="79"/>
-      <c r="G14" s="79"/>
-      <c r="H14" s="79"/>
-      <c r="I14" s="79"/>
-      <c r="J14" s="79"/>
-      <c r="K14" s="79"/>
-      <c r="L14" s="79"/>
-      <c r="M14" s="79"/>
-      <c r="N14" s="80"/>
+      <c r="C14" s="60"/>
+      <c r="D14" s="60"/>
+      <c r="E14" s="60"/>
+      <c r="F14" s="60"/>
+      <c r="G14" s="60"/>
+      <c r="H14" s="60"/>
+      <c r="I14" s="60"/>
+      <c r="J14" s="60"/>
+      <c r="K14" s="60"/>
+      <c r="L14" s="60"/>
+      <c r="M14" s="60"/>
+      <c r="N14" s="61"/>
     </row>
     <row r="15" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="59" t="s">
+      <c r="B15" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="C15" s="62" t="s">
+      <c r="C15" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="63"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="63"/>
-      <c r="G15" s="63"/>
-      <c r="H15" s="63"/>
-      <c r="I15" s="63"/>
-      <c r="J15" s="63"/>
-      <c r="K15" s="63"/>
-      <c r="L15" s="63"/>
-      <c r="M15" s="63"/>
-      <c r="N15" s="64"/>
+      <c r="D15" s="51"/>
+      <c r="E15" s="51"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="51"/>
+      <c r="H15" s="51"/>
+      <c r="I15" s="51"/>
+      <c r="J15" s="51"/>
+      <c r="K15" s="51"/>
+      <c r="L15" s="51"/>
+      <c r="M15" s="51"/>
+      <c r="N15" s="52"/>
     </row>
     <row r="16" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="81"/>
-      <c r="C16" s="65">
+      <c r="B16" s="48"/>
+      <c r="C16" s="53">
         <v>500</v>
       </c>
-      <c r="D16" s="66"/>
-      <c r="E16" s="67"/>
-      <c r="F16" s="68">
+      <c r="D16" s="54"/>
+      <c r="E16" s="55"/>
+      <c r="F16" s="56">
         <v>1000</v>
       </c>
-      <c r="G16" s="69"/>
-      <c r="H16" s="70"/>
-      <c r="I16" s="65">
+      <c r="G16" s="57"/>
+      <c r="H16" s="58"/>
+      <c r="I16" s="53">
         <v>2000</v>
       </c>
-      <c r="J16" s="66"/>
-      <c r="K16" s="67"/>
-      <c r="L16" s="83">
+      <c r="J16" s="54"/>
+      <c r="K16" s="55"/>
+      <c r="L16" s="62">
         <v>5000</v>
       </c>
-      <c r="M16" s="69"/>
-      <c r="N16" s="70"/>
+      <c r="M16" s="57"/>
+      <c r="N16" s="58"/>
     </row>
     <row r="17" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="82"/>
+      <c r="B17" s="49"/>
       <c r="C17" s="2" t="s">
         <v>3</v>
       </c>
@@ -15187,8 +15187,8 @@
         <v>1.9646539027982326</v>
       </c>
       <c r="K19" s="12">
-        <f xml:space="preserve"> J19 / 4</f>
-        <v>0.49116347569955815</v>
+        <f xml:space="preserve"> J19 / 2</f>
+        <v>0.9823269513991163</v>
       </c>
       <c r="L19" s="24">
         <v>3.4990000000000001</v>
@@ -15236,8 +15236,8 @@
         <v>3.6102841677943167</v>
       </c>
       <c r="K20" s="16">
-        <f xml:space="preserve"> J20 / 8</f>
-        <v>0.45128552097428959</v>
+        <f xml:space="preserve"> J20 / 4</f>
+        <v>0.90257104194857918</v>
       </c>
       <c r="L20" s="26">
         <v>1.9219999999999999</v>
@@ -15285,8 +15285,8 @@
         <v>6.4914841849148424</v>
       </c>
       <c r="K21" s="12">
-        <f xml:space="preserve"> J21 / 12</f>
-        <v>0.5409570154095702</v>
+        <f xml:space="preserve"> J21 / 8</f>
+        <v>0.81143552311435529</v>
       </c>
       <c r="L21" s="24">
         <v>1.024</v>
@@ -15334,8 +15334,8 @@
         <v>8.634304207119742</v>
       </c>
       <c r="K22" s="16">
-        <f xml:space="preserve"> J22 / 16</f>
-        <v>0.53964401294498388</v>
+        <f xml:space="preserve"> J22 / 12</f>
+        <v>0.7195253505933118</v>
       </c>
       <c r="L22" s="26">
         <v>0.77300000000000002</v>
@@ -15400,66 +15400,66 @@
     </row>
     <row r="24" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="25" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="71" t="s">
+      <c r="B25" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="C25" s="72"/>
-      <c r="D25" s="72"/>
-      <c r="E25" s="72"/>
-      <c r="F25" s="72"/>
-      <c r="G25" s="72"/>
-      <c r="H25" s="72"/>
-      <c r="I25" s="72"/>
-      <c r="J25" s="72"/>
-      <c r="K25" s="72"/>
-      <c r="L25" s="72"/>
-      <c r="M25" s="72"/>
-      <c r="N25" s="73"/>
+      <c r="C25" s="64"/>
+      <c r="D25" s="64"/>
+      <c r="E25" s="64"/>
+      <c r="F25" s="64"/>
+      <c r="G25" s="64"/>
+      <c r="H25" s="64"/>
+      <c r="I25" s="64"/>
+      <c r="J25" s="64"/>
+      <c r="K25" s="64"/>
+      <c r="L25" s="64"/>
+      <c r="M25" s="64"/>
+      <c r="N25" s="65"/>
     </row>
     <row r="26" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="74" t="s">
+      <c r="B26" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="C26" s="62" t="s">
+      <c r="C26" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="D26" s="63"/>
-      <c r="E26" s="63"/>
-      <c r="F26" s="63"/>
-      <c r="G26" s="63"/>
-      <c r="H26" s="63"/>
-      <c r="I26" s="63"/>
-      <c r="J26" s="63"/>
-      <c r="K26" s="63"/>
-      <c r="L26" s="63"/>
-      <c r="M26" s="63"/>
-      <c r="N26" s="64"/>
+      <c r="D26" s="51"/>
+      <c r="E26" s="51"/>
+      <c r="F26" s="51"/>
+      <c r="G26" s="51"/>
+      <c r="H26" s="51"/>
+      <c r="I26" s="51"/>
+      <c r="J26" s="51"/>
+      <c r="K26" s="51"/>
+      <c r="L26" s="51"/>
+      <c r="M26" s="51"/>
+      <c r="N26" s="52"/>
     </row>
     <row r="27" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="60"/>
-      <c r="C27" s="65">
+      <c r="B27" s="67"/>
+      <c r="C27" s="53">
         <v>500</v>
       </c>
-      <c r="D27" s="66"/>
-      <c r="E27" s="67"/>
-      <c r="F27" s="68">
+      <c r="D27" s="54"/>
+      <c r="E27" s="55"/>
+      <c r="F27" s="56">
         <v>1000</v>
       </c>
-      <c r="G27" s="69"/>
-      <c r="H27" s="70"/>
-      <c r="I27" s="65">
+      <c r="G27" s="57"/>
+      <c r="H27" s="58"/>
+      <c r="I27" s="53">
         <v>2000</v>
       </c>
-      <c r="J27" s="66"/>
-      <c r="K27" s="67"/>
-      <c r="L27" s="75">
+      <c r="J27" s="54"/>
+      <c r="K27" s="55"/>
+      <c r="L27" s="69">
         <v>5000</v>
       </c>
-      <c r="M27" s="76"/>
-      <c r="N27" s="77"/>
+      <c r="M27" s="70"/>
+      <c r="N27" s="71"/>
     </row>
     <row r="28" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="61"/>
+      <c r="B28" s="68"/>
       <c r="C28" s="2" t="s">
         <v>3</v>
       </c>
@@ -15577,8 +15577,8 @@
         <v>2.0652622883106155</v>
       </c>
       <c r="K30" s="12">
-        <f xml:space="preserve"> J30 / 4</f>
-        <v>0.51631557207765388</v>
+        <f xml:space="preserve"> J30 / 2</f>
+        <v>1.0326311441553078</v>
       </c>
       <c r="L30" s="10">
         <v>6.1760000000000002</v>
@@ -15626,8 +15626,8 @@
         <v>3.8610038610038613</v>
       </c>
       <c r="K31" s="16">
-        <f xml:space="preserve"> J31 / 8</f>
-        <v>0.48262548262548266</v>
+        <f xml:space="preserve"> J31 / 4</f>
+        <v>0.96525096525096532</v>
       </c>
       <c r="L31" s="14">
         <v>3.2679999999999998</v>
@@ -15675,8 +15675,8 @@
         <v>6.4516129032258061</v>
       </c>
       <c r="K32" s="12">
-        <f xml:space="preserve"> J32 / 12</f>
-        <v>0.5376344086021505</v>
+        <f xml:space="preserve"> J32 / 8</f>
+        <v>0.80645161290322576</v>
       </c>
       <c r="L32" s="10">
         <v>1.823</v>
@@ -15724,8 +15724,8 @@
         <v>8.9928057553956826</v>
       </c>
       <c r="K33" s="16">
-        <f xml:space="preserve"> J33 / 16</f>
-        <v>0.56205035971223016</v>
+        <f xml:space="preserve"> J33 / 12</f>
+        <v>0.74940047961630685</v>
       </c>
       <c r="L33" s="14">
         <v>1.385</v>
@@ -15790,66 +15790,66 @@
     </row>
     <row r="35" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="36" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="56" t="s">
+      <c r="B36" s="72" t="s">
         <v>14</v>
       </c>
-      <c r="C36" s="57"/>
-      <c r="D36" s="57"/>
-      <c r="E36" s="57"/>
-      <c r="F36" s="57"/>
-      <c r="G36" s="57"/>
-      <c r="H36" s="57"/>
-      <c r="I36" s="57"/>
-      <c r="J36" s="57"/>
-      <c r="K36" s="57"/>
-      <c r="L36" s="57"/>
-      <c r="M36" s="57"/>
-      <c r="N36" s="58"/>
+      <c r="C36" s="73"/>
+      <c r="D36" s="73"/>
+      <c r="E36" s="73"/>
+      <c r="F36" s="73"/>
+      <c r="G36" s="73"/>
+      <c r="H36" s="73"/>
+      <c r="I36" s="73"/>
+      <c r="J36" s="73"/>
+      <c r="K36" s="73"/>
+      <c r="L36" s="73"/>
+      <c r="M36" s="73"/>
+      <c r="N36" s="74"/>
     </row>
     <row r="37" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="59" t="s">
+      <c r="B37" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="C37" s="62" t="s">
+      <c r="C37" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="D37" s="63"/>
-      <c r="E37" s="63"/>
-      <c r="F37" s="63"/>
-      <c r="G37" s="63"/>
-      <c r="H37" s="63"/>
-      <c r="I37" s="63"/>
-      <c r="J37" s="63"/>
-      <c r="K37" s="63"/>
-      <c r="L37" s="63"/>
-      <c r="M37" s="63"/>
-      <c r="N37" s="64"/>
+      <c r="D37" s="51"/>
+      <c r="E37" s="51"/>
+      <c r="F37" s="51"/>
+      <c r="G37" s="51"/>
+      <c r="H37" s="51"/>
+      <c r="I37" s="51"/>
+      <c r="J37" s="51"/>
+      <c r="K37" s="51"/>
+      <c r="L37" s="51"/>
+      <c r="M37" s="51"/>
+      <c r="N37" s="52"/>
     </row>
     <row r="38" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="60"/>
-      <c r="C38" s="65">
+      <c r="B38" s="67"/>
+      <c r="C38" s="53">
         <v>500</v>
       </c>
-      <c r="D38" s="66"/>
-      <c r="E38" s="67"/>
-      <c r="F38" s="68">
+      <c r="D38" s="54"/>
+      <c r="E38" s="55"/>
+      <c r="F38" s="56">
         <v>1000</v>
       </c>
-      <c r="G38" s="69"/>
-      <c r="H38" s="70"/>
-      <c r="I38" s="65">
+      <c r="G38" s="57"/>
+      <c r="H38" s="58"/>
+      <c r="I38" s="53">
         <v>2000</v>
       </c>
-      <c r="J38" s="66"/>
-      <c r="K38" s="67"/>
-      <c r="L38" s="68">
+      <c r="J38" s="54"/>
+      <c r="K38" s="55"/>
+      <c r="L38" s="56">
         <v>5000</v>
       </c>
-      <c r="M38" s="69"/>
-      <c r="N38" s="70"/>
+      <c r="M38" s="57"/>
+      <c r="N38" s="58"/>
     </row>
     <row r="39" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="61"/>
+      <c r="B39" s="68"/>
       <c r="C39" s="2" t="s">
         <v>3</v>
       </c>
@@ -15967,8 +15967,8 @@
         <v>1.9519497320273518</v>
       </c>
       <c r="K41" s="37">
-        <f xml:space="preserve"> J41 / 4</f>
-        <v>0.48798743300683795</v>
+        <f xml:space="preserve"> J41 / 2</f>
+        <v>0.97597486601367589</v>
       </c>
       <c r="L41" s="10">
         <v>13.872999999999999</v>
@@ -16016,8 +16016,8 @@
         <v>3.7007708479327257</v>
       </c>
       <c r="K42" s="37">
-        <f xml:space="preserve"> J42 / 8</f>
-        <v>0.46259635599159071</v>
+        <f xml:space="preserve"> J42 / 4</f>
+        <v>0.92519271198318143</v>
       </c>
       <c r="L42" s="14">
         <v>7.16</v>
@@ -16065,8 +16065,8 @@
         <v>6.4678505817513772</v>
       </c>
       <c r="K43" s="37">
-        <f xml:space="preserve"> J43 / 12</f>
-        <v>0.53898754847928143</v>
+        <f xml:space="preserve"> J43 / 8</f>
+        <v>0.80848132271892215</v>
       </c>
       <c r="L43" s="10">
         <v>4.0019999999999998</v>
@@ -16114,8 +16114,8 @@
         <v>8.9736618521665239</v>
       </c>
       <c r="K44" s="37">
-        <f xml:space="preserve"> J44 / 16</f>
-        <v>0.56085386576040774</v>
+        <f xml:space="preserve"> J44 / 12</f>
+        <v>0.74780515434721029</v>
       </c>
       <c r="L44" s="14">
         <v>3.0739999999999998</v>
@@ -16180,70 +16180,96 @@
     </row>
     <row r="46" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="47" spans="2:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B47" s="44" t="s">
+      <c r="B47" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C47" s="45"/>
-      <c r="D47" s="45"/>
-      <c r="E47" s="45"/>
-      <c r="F47" s="45"/>
-      <c r="G47" s="45"/>
-      <c r="H47" s="46"/>
+      <c r="C47" s="76"/>
+      <c r="D47" s="76"/>
+      <c r="E47" s="76"/>
+      <c r="F47" s="76"/>
+      <c r="G47" s="76"/>
+      <c r="H47" s="77"/>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B48" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="C48" s="47" t="s">
+      <c r="C48" s="78" t="s">
         <v>17</v>
       </c>
-      <c r="D48" s="48"/>
-      <c r="E48" s="48"/>
-      <c r="F48" s="48"/>
-      <c r="G48" s="48"/>
-      <c r="H48" s="49"/>
+      <c r="D48" s="79"/>
+      <c r="E48" s="79"/>
+      <c r="F48" s="79"/>
+      <c r="G48" s="79"/>
+      <c r="H48" s="80"/>
     </row>
     <row r="49" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B49" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="C49" s="50" t="s">
+      <c r="C49" s="81" t="s">
         <v>19</v>
       </c>
-      <c r="D49" s="51"/>
-      <c r="E49" s="51"/>
-      <c r="F49" s="51"/>
-      <c r="G49" s="51"/>
-      <c r="H49" s="52"/>
+      <c r="D49" s="82"/>
+      <c r="E49" s="82"/>
+      <c r="F49" s="82"/>
+      <c r="G49" s="82"/>
+      <c r="H49" s="83"/>
     </row>
     <row r="50" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B50" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="C50" s="50" t="s">
+      <c r="C50" s="81" t="s">
         <v>21</v>
       </c>
-      <c r="D50" s="51"/>
-      <c r="E50" s="51"/>
-      <c r="F50" s="51"/>
-      <c r="G50" s="51"/>
-      <c r="H50" s="52"/>
+      <c r="D50" s="82"/>
+      <c r="E50" s="82"/>
+      <c r="F50" s="82"/>
+      <c r="G50" s="82"/>
+      <c r="H50" s="83"/>
     </row>
     <row r="51" spans="2:8" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B51" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="C51" s="53" t="s">
+      <c r="C51" s="84" t="s">
         <v>23</v>
       </c>
-      <c r="D51" s="54"/>
-      <c r="E51" s="54"/>
-      <c r="F51" s="54"/>
-      <c r="G51" s="54"/>
-      <c r="H51" s="55"/>
+      <c r="D51" s="85"/>
+      <c r="E51" s="85"/>
+      <c r="F51" s="85"/>
+      <c r="G51" s="85"/>
+      <c r="H51" s="86"/>
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="B47:H47"/>
+    <mergeCell ref="C48:H48"/>
+    <mergeCell ref="C49:H49"/>
+    <mergeCell ref="C50:H50"/>
+    <mergeCell ref="C51:H51"/>
+    <mergeCell ref="B36:N36"/>
+    <mergeCell ref="B37:B39"/>
+    <mergeCell ref="C37:N37"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="F38:H38"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="L38:N38"/>
+    <mergeCell ref="B25:N25"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="C26:N26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="F27:H27"/>
+    <mergeCell ref="I27:K27"/>
+    <mergeCell ref="L27:N27"/>
+    <mergeCell ref="B14:N14"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="C15:N15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="L16:N16"/>
     <mergeCell ref="B3:N3"/>
     <mergeCell ref="B4:B6"/>
     <mergeCell ref="C4:N4"/>
@@ -16251,32 +16277,6 @@
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="I5:K5"/>
     <mergeCell ref="L5:N5"/>
-    <mergeCell ref="B14:N14"/>
-    <mergeCell ref="B15:B17"/>
-    <mergeCell ref="C15:N15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="F16:H16"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="L16:N16"/>
-    <mergeCell ref="B25:N25"/>
-    <mergeCell ref="B26:B28"/>
-    <mergeCell ref="C26:N26"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="F27:H27"/>
-    <mergeCell ref="I27:K27"/>
-    <mergeCell ref="L27:N27"/>
-    <mergeCell ref="B36:N36"/>
-    <mergeCell ref="B37:B39"/>
-    <mergeCell ref="C37:N37"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="F38:H38"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="L38:N38"/>
-    <mergeCell ref="B47:H47"/>
-    <mergeCell ref="C48:H48"/>
-    <mergeCell ref="C49:H49"/>
-    <mergeCell ref="C50:H50"/>
-    <mergeCell ref="C51:H51"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>